<commit_message>
evaluated agent on validation and testing data
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muneebmuhammad/Documents/masters/sem 1/AI Systems/GPU-Broker/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55FE724B-9BB8-F848-8E4B-AFD15586E21A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{794A200C-E232-5C46-94E0-1FA5AD84ED8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="223">
   <si>
     <t>input_text</t>
   </si>
@@ -374,9 +374,6 @@
     <t>Do not use LoRA or QLoRA. Fully fine-tune Llama 3.2 1B on 3 GB of text using sequence length 1024, batch size 8, FP16, and 2 epochs. Training must finish in 5 hours.</t>
   </si>
   <si>
-    <t>I need two jobs for Llama 3.2 3B: LoRA training on a 5 GB dataset, and a separate inference endpoint. I have not chosen which job this request should represent.</t>
-  </si>
-  <si>
     <t>LoRA-tune Mistral 7B on 4 GB of text with sequence length 2048, batch size 0, BF16 precision, and 2 epochs.</t>
   </si>
   <si>
@@ -680,9 +677,6 @@
     <t>Negation: Explicitly requested full update overrides negated LoRA/QLoRA.</t>
   </si>
   <si>
-    <t>Mixed workload: Single row cannot represent training and inference; retain common model fields and clarify/split jobs.</t>
-  </si>
-  <si>
     <t>Invalid value: Extraction preserves the stated zero; validation must reject it, not silently replace it.</t>
   </si>
   <si>
@@ -690,6 +684,12 @@
   </si>
   <si>
     <t>I want to fine-tune Llama 3.2 3B using  LoRA on a 50 GB text dataset. I plan to use a sequence length of 2048, batch  size of 8, BF16 precision, and train for 3 epochs.</t>
+  </si>
+  <si>
+    <t>I need a jobs for Llama 3.2 3B: LoRA training on a 5 GB dataset.</t>
+  </si>
+  <si>
+    <t>Missing fields: Sequence length missing.</t>
   </si>
 </sst>
 </file>
@@ -1066,7 +1066,7 @@
     </row>
     <row r="2" spans="1:13" ht="40" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>13</v>
@@ -1107,7 +1107,7 @@
     </row>
     <row r="3" spans="1:13" ht="40" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>18</v>
@@ -1780,8 +1780,8 @@
       <c r="F19" s="5">
         <v>8</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>40</v>
+      <c r="G19" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="H19" s="1" t="s">
         <v>20</v>
@@ -3010,8 +3010,8 @@
       <c r="F49" s="5">
         <v>8</v>
       </c>
-      <c r="G49" s="1" t="s">
-        <v>40</v>
+      <c r="G49" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="H49" s="1" t="s">
         <v>20</v>
@@ -3444,7 +3444,7 @@
     </row>
     <row r="60" spans="1:13" ht="40" customHeight="1">
       <c r="A60" s="3" t="s">
-        <v>117</v>
+        <v>221</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>18</v>
@@ -3452,8 +3452,8 @@
       <c r="C60" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D60" s="4" t="s">
-        <v>15</v>
+      <c r="D60" s="4">
+        <v>5</v>
       </c>
       <c r="E60" s="4" t="s">
         <v>15</v>
@@ -3461,8 +3461,8 @@
       <c r="F60" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G60" s="3" t="s">
-        <v>15</v>
+      <c r="G60" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="H60" s="3" t="s">
         <v>15</v>
@@ -3479,13 +3479,13 @@
       <c r="L60" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="M60" s="3" t="s">
-        <v>15</v>
+      <c r="M60" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="61" spans="1:13" ht="40" customHeight="1">
       <c r="A61" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>29</v>
@@ -3543,170 +3543,170 @@
   <sheetData>
     <row r="1" spans="1:2" ht="25" customHeight="1">
       <c r="A1" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="38" customHeight="1">
       <c r="A2" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="38" customHeight="1">
       <c r="A3" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="52" customHeight="1">
       <c r="A4" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="52" customHeight="1">
       <c r="A5" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="38" customHeight="1">
       <c r="A6" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="38" customHeight="1">
       <c r="A7" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="38" customHeight="1">
       <c r="A8" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="52" customHeight="1">
       <c r="A9" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="52" customHeight="1">
       <c r="A10" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="52" customHeight="1">
       <c r="A11" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="38" customHeight="1">
       <c r="A12" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="80" customHeight="1">
       <c r="A13" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="52" customHeight="1">
       <c r="A14" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="38" customHeight="1">
       <c r="A15" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="38" customHeight="1">
       <c r="A16" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="52" customHeight="1">
       <c r="A17" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="52" customHeight="1">
       <c r="A18" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="52" customHeight="1">
       <c r="A19" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="52" customHeight="1">
       <c r="A20" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="25" customHeight="1">
       <c r="A21" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>159</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="32" customHeight="1">
@@ -3714,7 +3714,7 @@
         <v>1</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="32" customHeight="1">
@@ -3722,7 +3722,7 @@
         <v>2</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="32" customHeight="1">
@@ -3730,7 +3730,7 @@
         <v>3</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="32" customHeight="1">
@@ -3738,7 +3738,7 @@
         <v>4</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="32" customHeight="1">
@@ -3746,7 +3746,7 @@
         <v>5</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="32" customHeight="1">
@@ -3754,7 +3754,7 @@
         <v>6</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="32" customHeight="1">
@@ -3762,7 +3762,7 @@
         <v>7</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="32" customHeight="1">
@@ -3770,7 +3770,7 @@
         <v>8</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="32" customHeight="1">
@@ -3778,7 +3778,7 @@
         <v>9</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="32" customHeight="1">
@@ -3786,7 +3786,7 @@
         <v>10</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="32" customHeight="1">
@@ -3794,7 +3794,7 @@
         <v>11</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="32" customHeight="1">
@@ -3802,7 +3802,7 @@
         <v>12</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="32" customHeight="1">
@@ -3810,7 +3810,7 @@
         <v>13</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="32" customHeight="1">
@@ -3818,7 +3818,7 @@
         <v>14</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="32" customHeight="1">
@@ -3826,7 +3826,7 @@
         <v>15</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="32" customHeight="1">
@@ -3834,7 +3834,7 @@
         <v>16</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="32" customHeight="1">
@@ -3842,7 +3842,7 @@
         <v>17</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="32" customHeight="1">
@@ -3850,7 +3850,7 @@
         <v>18</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="32" customHeight="1">
@@ -3858,7 +3858,7 @@
         <v>19</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="32" customHeight="1">
@@ -3866,7 +3866,7 @@
         <v>20</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="32" customHeight="1">
@@ -3874,7 +3874,7 @@
         <v>21</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="32" customHeight="1">
@@ -3882,7 +3882,7 @@
         <v>22</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="32" customHeight="1">
@@ -3890,7 +3890,7 @@
         <v>23</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="32" customHeight="1">
@@ -3898,7 +3898,7 @@
         <v>24</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="32" customHeight="1">
@@ -3906,7 +3906,7 @@
         <v>25</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="32" customHeight="1">
@@ -3914,7 +3914,7 @@
         <v>26</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="32" customHeight="1">
@@ -3922,7 +3922,7 @@
         <v>27</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="32" customHeight="1">
@@ -3930,7 +3930,7 @@
         <v>28</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="32" customHeight="1">
@@ -3938,7 +3938,7 @@
         <v>29</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="32" customHeight="1">
@@ -3946,7 +3946,7 @@
         <v>30</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="32" customHeight="1">
@@ -3954,7 +3954,7 @@
         <v>31</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="32" customHeight="1">
@@ -3962,7 +3962,7 @@
         <v>32</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="32" customHeight="1">
@@ -3970,7 +3970,7 @@
         <v>33</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="32" customHeight="1">
@@ -3978,7 +3978,7 @@
         <v>34</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="32" customHeight="1">
@@ -3986,7 +3986,7 @@
         <v>35</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="32" customHeight="1">
@@ -3994,7 +3994,7 @@
         <v>36</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="32" customHeight="1">
@@ -4002,7 +4002,7 @@
         <v>37</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="32" customHeight="1">
@@ -4010,7 +4010,7 @@
         <v>38</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="32" customHeight="1">
@@ -4018,7 +4018,7 @@
         <v>39</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="32" customHeight="1">
@@ -4026,7 +4026,7 @@
         <v>40</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="32" customHeight="1">
@@ -4034,7 +4034,7 @@
         <v>41</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="32" customHeight="1">
@@ -4042,7 +4042,7 @@
         <v>42</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="32" customHeight="1">
@@ -4050,7 +4050,7 @@
         <v>43</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="32" customHeight="1">
@@ -4058,7 +4058,7 @@
         <v>44</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="32" customHeight="1">
@@ -4066,7 +4066,7 @@
         <v>45</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="32" customHeight="1">
@@ -4074,7 +4074,7 @@
         <v>46</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="32" customHeight="1">
@@ -4082,7 +4082,7 @@
         <v>47</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="32" customHeight="1">
@@ -4090,7 +4090,7 @@
         <v>48</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="32" customHeight="1">
@@ -4098,7 +4098,7 @@
         <v>49</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="38" customHeight="1">
@@ -4106,7 +4106,7 @@
         <v>50</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="32" customHeight="1">
@@ -4114,7 +4114,7 @@
         <v>51</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="32" customHeight="1">
@@ -4122,7 +4122,7 @@
         <v>52</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="32" customHeight="1">
@@ -4130,7 +4130,7 @@
         <v>53</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="32" customHeight="1">
@@ -4138,7 +4138,7 @@
         <v>54</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="32" customHeight="1">
@@ -4146,7 +4146,7 @@
         <v>55</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="32" customHeight="1">
@@ -4154,7 +4154,7 @@
         <v>56</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="32" customHeight="1">
@@ -4162,7 +4162,7 @@
         <v>57</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="32" customHeight="1">
@@ -4170,7 +4170,7 @@
         <v>58</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="32" customHeight="1">
@@ -4178,7 +4178,7 @@
         <v>59</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="32" customHeight="1">
@@ -4186,7 +4186,7 @@
         <v>60</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>